<commit_message>
Add Control entries to the cronograma alongside each tarea due date
One control per tarea (5 total), same day the tarea is handed in,
matching the new "Tareas y controles" policy in the syllabus.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cronograma_Analisis_Econometrico_2026.xlsx
+++ b/Cronograma_Analisis_Econometrico_2026.xlsx
@@ -742,7 +742,7 @@
       <c r="E12" s="16" t="n"/>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Tarea 1</t>
+          <t>Tarea 1 / Control 1</t>
         </is>
       </c>
       <c r="G12" s="13" t="n"/>
@@ -925,7 +925,7 @@
       <c r="E21" s="16" t="n"/>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Tarea 2</t>
+          <t>Tarea 2 / Control 2</t>
         </is>
       </c>
       <c r="G21" s="13" t="n"/>
@@ -1112,7 +1112,7 @@
       <c r="E30" s="16" t="n"/>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Tarea 3</t>
+          <t>Tarea 3 / Control 3</t>
         </is>
       </c>
       <c r="G30" s="13" t="n"/>
@@ -1294,7 +1294,7 @@
       <c r="E39" s="16" t="n"/>
       <c r="F39" s="13" t="inlineStr">
         <is>
-          <t>Tarea 4</t>
+          <t>Tarea 4 / Control 4</t>
         </is>
       </c>
       <c r="G39" s="13" t="n"/>
@@ -1435,7 +1435,7 @@
       <c r="E46" s="3" t="n"/>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Tarea 5</t>
+          <t>Tarea 5 / Control 5</t>
         </is>
       </c>
       <c r="G46" s="5" t="n"/>

</xml_diff>